<commit_message>
deleted db fields timezone, location, routing. Replaced in sheet params of xlxs in db
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -8,9 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="default" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="replacement" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="inside" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="default" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="replacement" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="inside" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,15 +23,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timezon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europe/Paris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">routing</t>
+  </si>
   <si>
     <t xml:space="preserve">table</t>
   </si>
   <si>
     <t xml:space="preserve">field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value</t>
   </si>
   <si>
     <t xml:space="preserve">type</t>
@@ -176,7 +192,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -303,49 +319,39 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B3" s="1" t="n">
+        <v>1396</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>9</v>
+      <c r="B4" s="1" t="n">
+        <v>7012</v>
       </c>
     </row>
   </sheetData>
@@ -364,45 +370,106 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="0" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>15</v>
+        <v>19</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -416,7 +483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -425,36 +492,36 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="0" t="s">
-        <v>20</v>
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>23</v>
+      <c r="A2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>23</v>
+      <c r="A3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new state created : save_db
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -9,9 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="default" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="replacement" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="inside" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="replacement" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="inside" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -40,34 +39,13 @@
     <t xml:space="preserve">location</t>
   </si>
   <si>
-    <t xml:space="preserve">routing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timetables</t>
-  </si>
-  <si>
     <t xml:space="preserve">gong_id</t>
   </si>
   <si>
-    <t xml:space="preserve">int</t>
-  </si>
-  <si>
     <t xml:space="preserve">targets</t>
   </si>
   <si>
     <t xml:space="preserve">CC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">str</t>
   </si>
   <si>
     <t xml:space="preserve">period_type</t>
@@ -319,7 +297,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -351,8 +329,20 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>7012</v>
-      </c>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -366,67 +356,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -441,35 +370,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -483,7 +412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -493,35 +422,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
default period in pexcel params + OK overlap in plan
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -48,6 +48,12 @@
     <t xml:space="preserve">CC</t>
   </si>
   <si>
+    <t xml:space="preserve">default_period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN BETWEEN</t>
+  </si>
+  <si>
     <t xml:space="preserve">period_type</t>
   </si>
   <si>
@@ -64,9 +70,6 @@
   </si>
   <si>
     <t xml:space="preserve">TRUSTMEETING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN BETWEEN</t>
   </si>
   <si>
     <t xml:space="preserve">ServicePeriod</t>
@@ -341,8 +344,12 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -370,35 +377,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -422,46 +429,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="1" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>14</v>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
before calculating durationd FROM minio
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -197,37 +197,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -332,7 +332,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
fixed: start date of plan + show 'no-gong' periods
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -424,8 +424,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.91"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -468,6 +471,17 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
insert 'Service d0' before 'Service after d0'
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -84,6 +84,9 @@
     <t xml:space="preserve">container</t>
   </si>
   <si>
+    <t xml:space="preserve">after</t>
+  </si>
+  <si>
     <t xml:space="preserve">delete</t>
   </si>
   <si>
@@ -94,6 +97,15 @@
   </si>
   <si>
     <t xml:space="preserve">Children / teens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service d0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service after d0</t>
   </si>
 </sst>
 </file>
@@ -168,12 +180,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -424,10 +440,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -440,35 +457,38 @@
       <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="D1" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>9</v>
@@ -476,13 +496,27 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
help text + tighter timings + timing trace
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -84,9 +84,6 @@
     <t xml:space="preserve">container</t>
   </si>
   <si>
-    <t xml:space="preserve">after</t>
-  </si>
-  <si>
     <t xml:space="preserve">delete</t>
   </si>
   <si>
@@ -97,15 +94,6 @@
   </si>
   <si>
     <t xml:space="preserve">Children / teens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insert1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service d0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service after d0</t>
   </si>
 </sst>
 </file>
@@ -180,16 +168,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -213,37 +197,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -348,7 +332,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -440,12 +424,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.63"/>
-  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -457,66 +437,38 @@
       <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="0" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
blockquote in utils.py, no more in markdown text
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -93,16 +93,16 @@
     <t xml:space="preserve">1 day</t>
   </si>
   <si>
+    <t xml:space="preserve">Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Children / teens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Service d0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Children / teens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insert1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service</t>
   </si>
   <si>
     <t xml:space="preserve">Service after d0</t>
@@ -213,37 +213,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -444,7 +444,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -457,7 +457,7 @@
       <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="0" t="s">
         <v>20</v>
       </c>
     </row>
@@ -468,7 +468,7 @@
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -479,7 +479,7 @@
       <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -510,12 +510,12 @@
         <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="0" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Testx OK with/without confirmation
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -93,16 +93,16 @@
     <t xml:space="preserve">1 day</t>
   </si>
   <si>
+    <t xml:space="preserve">Service d0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Children / teens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Children / teens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insert1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service d0</t>
   </si>
   <si>
     <t xml:space="preserve">Service after d0</t>
@@ -213,37 +213,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -444,7 +444,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -457,7 +457,7 @@
       <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -468,7 +468,7 @@
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -479,7 +479,7 @@
       <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -510,12 +510,12 @@
         <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="2" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
corrected updating model attribute + listener on-transition (and NOT after)
</commit_message>
<xml_diff>
--- a/data/Mahi.xlsx
+++ b/data/Mahi.xlsx
@@ -93,16 +93,16 @@
     <t xml:space="preserve">1 day</t>
   </si>
   <si>
+    <t xml:space="preserve">Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Children / teens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Service d0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Children / teens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insert1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service</t>
   </si>
   <si>
     <t xml:space="preserve">Service after d0</t>
@@ -213,37 +213,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -444,7 +444,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -457,7 +457,7 @@
       <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="0" t="s">
         <v>20</v>
       </c>
     </row>
@@ -468,7 +468,7 @@
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -479,7 +479,7 @@
       <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -510,12 +510,12 @@
         <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="0" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>